<commit_message>
ci: add playwright tests and github actions automation workflow
</commit_message>
<xml_diff>
--- a/smart_travel_planner_test_case_report.xlsx
+++ b/smart_travel_planner_test_case_report.xlsx
@@ -520,43 +520,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Module / Component</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Test Title</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Preconditions</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
     <row r="3" ht="10" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -4379,43 +4343,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Module / Component</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Test Title</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Preconditions</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
+    <row r="2"/>
     <row r="3" ht="10" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="n"/>

</xml_diff>